<commit_message>
Initial commit - GridSentinel AI project
</commit_message>
<xml_diff>
--- a/data/audit_log.xlsx
+++ b/data/audit_log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="9">
   <si>
     <t>timestamp</t>
   </si>
@@ -25,7 +25,7 @@
     <t>action</t>
   </si>
   <si>
-    <t>engineer@bescom.co.in</t>
+    <t>admin@bescom.in</t>
   </si>
   <si>
     <t>LOGIN</t>
@@ -35,6 +35,12 @@
   </si>
   <si>
     <t>VIEW_CHARTS</t>
+  </si>
+  <si>
+    <t>VIEW_ADMIN</t>
+  </si>
+  <si>
+    <t>LOGOUT</t>
   </si>
 </sst>
 </file>
@@ -396,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -412,7 +418,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2">
-        <v>46141.75636018519</v>
+        <v>46149.83500083334</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -423,134 +429,68 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2">
-        <v>46141.75881362268</v>
+        <v>46149.83501875</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="2">
-        <v>46141.76150335648</v>
+        <v>46149.83517824074</v>
       </c>
       <c r="B4" t="s">
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="2">
-        <v>46141.76151508102</v>
+        <v>46149.83521923611</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="2">
-        <v>46141.76159385416</v>
+        <v>46149.8353316088</v>
       </c>
       <c r="B6" t="s">
         <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="2">
-        <v>46141.7616569213</v>
+        <v>46149.83571891204</v>
       </c>
       <c r="B7" t="s">
         <v>3</v>
       </c>
       <c r="C7" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="2">
-        <v>46141.76235835648</v>
+        <v>46149.83582451918</v>
       </c>
       <c r="B8" t="s">
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" s="2">
-        <v>46141.76239885417</v>
-      </c>
-      <c r="B9" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" s="2">
-        <v>46141.76277296296</v>
-      </c>
-      <c r="B10" t="s">
-        <v>3</v>
-      </c>
-      <c r="C10" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="2">
-        <v>46141.76282166666</v>
-      </c>
-      <c r="B11" t="s">
-        <v>3</v>
-      </c>
-      <c r="C11" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" s="2">
-        <v>46141.76285591435</v>
-      </c>
-      <c r="B12" t="s">
-        <v>3</v>
-      </c>
-      <c r="C12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" s="2">
-        <v>46141.76287694444</v>
-      </c>
-      <c r="B13" t="s">
-        <v>3</v>
-      </c>
-      <c r="C13" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
-      <c r="A14" s="2">
-        <v>46141.76290257757</v>
-      </c>
-      <c r="B14" t="s">
-        <v>3</v>
-      </c>
-      <c r="C14" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Initial commit - GridSentinel AI
</commit_message>
<xml_diff>
--- a/data/audit_log.xlsx
+++ b/data/audit_log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="7">
   <si>
     <t>timestamp</t>
   </si>
@@ -25,16 +25,10 @@
     <t>action</t>
   </si>
   <si>
-    <t>admin@bescom.in</t>
-  </si>
-  <si>
-    <t>LOGIN</t>
+    <t>Jitesh@bescom.in</t>
   </si>
   <si>
     <t>VIEW_DASHBOARD</t>
-  </si>
-  <si>
-    <t>VIEW_CHARTS</t>
   </si>
   <si>
     <t>VIEW_ADMIN</t>
@@ -402,7 +396,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -418,7 +412,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2">
-        <v>46149.83500083334</v>
+        <v>46149.86995635417</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -429,7 +423,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2">
-        <v>46149.83501875</v>
+        <v>46149.87023376158</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
@@ -440,7 +434,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="2">
-        <v>46149.83517824074</v>
+        <v>46149.87028121528</v>
       </c>
       <c r="B4" t="s">
         <v>3</v>
@@ -451,46 +445,24 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="2">
-        <v>46149.83521923611</v>
+        <v>46149.8705365625</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="2">
-        <v>46149.8353316088</v>
+        <v>46149.87060391397</v>
       </c>
       <c r="B6" t="s">
         <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="2">
-        <v>46149.83571891204</v>
-      </c>
-      <c r="B7" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="2">
-        <v>46149.83582451918</v>
-      </c>
-      <c r="B8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C8" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>